<commit_message>
audit and synchronize scenario 7 contracts
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Machine.xlsx
+++ b/Documentation/System_State_Machine.xlsx
@@ -13,11 +13,12 @@
     <sheet name="۳ حالت شارژر" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="۴ گذار شارژر" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="۵ خطاها" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="۶ چهرهٔ UI" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="۷ عدم‌توازن" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="۸ باتری خراب" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="۹ تغذیهٔ MCU" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="۱۰ لینک ESP" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="۵-الف خطای فنی" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="۶ چهرهٔ UI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="۷ عدم‌توازن" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="۸ باتری خراب" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="۹ تغذیهٔ MCU" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="۱۰ لینک ESP" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -76,6 +77,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
@@ -92,11 +98,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -529,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -647,94 +648,106 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>۶ چهرهٔ UI</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>اولویت سناریوها و چهرهٔ چراغ و بوق</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Firmware/Modules/Ui/ui_led.c</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>۵-الف خطای فنی</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>سناریوی ۷: تشخیص سوختن ترانزیستور، قفل RAM و reset</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/Charger/charger.c، Firmware/Modules/Ui/ui_led.c</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>۷ عدم‌توازن</t>
+          <t>۶ چهرهٔ UI</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>حالت‌های سناریوی ۵</t>
+          <t>اولویت سناریوها و چهرهٔ چراغ و بوق</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Firmware/Modules/Imbalance/imbalance.c</t>
+          <t>Firmware/Modules/Ui/ui_led.c</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>۸ باتری خراب</t>
+          <t>۷ عدم‌توازن</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>حالت‌های سناریوی ۶</t>
+          <t>حالت‌های سناریوی ۵</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>charger.c (DeadBatteryTick)</t>
+          <t>Firmware/Modules/Imbalance/imbalance.c</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>۹ تغذیهٔ MCU</t>
+          <t>۸ باتری خراب</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>مسیر تغذیهٔ خود میکرو</t>
+          <t>حالت‌های سناریوی ۶</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Firmware/Modules/McuPowerPath/mcu_power_path.c</t>
+          <t>charger.c (DeadBatteryTick)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>۹ تغذیهٔ MCU</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>مسیر تغذیهٔ خود میکرو</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/McuPowerPath/mcu_power_path.c</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>۱۰ لینک ESP</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>حالت پارسر و مراحل ارسال جدول</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Firmware/Modules/EspLink/esp_link.c، Firmware/Modules/CalLut/cal_lut.c</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr"/>
@@ -742,47 +755,52 @@
       <c r="C14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>نسخهٔ ماژولی</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>همین حالت‌ها، ماژول‌به‌ماژول و کنار برگهٔ اعتبارسنجی همان ماژول: Firmware/Modules/&lt;نام&gt;/&lt;نام&gt;_State_Machine.xlsx — برای کار روی میز تست از این‌ها استفاده کنید، این کتاب نمای سیستمی است</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>tools/make_module_state_machines.py</t>
-        </is>
-      </c>
+      <c r="A15" s="6" t="inlineStr"/>
+      <c r="B15" s="6" t="inlineStr"/>
+      <c r="C15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
+          <t>نسخهٔ ماژولی</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>همین حالت‌ها، ماژول‌به‌ماژول و کنار برگهٔ اعتبارسنجی همان ماژول: Firmware/Modules/&lt;نام&gt;/&lt;نام&gt;_State_Machine.xlsx — برای کار روی میز تست از این‌ها استفاده کنید، این کتاب نمای سیستمی است</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
           <t>رنگ‌ها</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>بازتولید</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>python3 tools/make_state_machine_xlsx.py</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>tools/make_state_machine_xlsx.py</t>
         </is>
@@ -797,6 +815,191 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ماشین حالت سناریوی ۶ (مهلت شارژ پیوسته)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>حالت</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>شرط ورود</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>شرط خروج</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>پارامترها</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>شمارش متوقف</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>کانال شارژ نمی‌کند</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>شروع BULK یا ABSORB</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>در حال شمارش</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>کانال در BULK یا ABSORB است</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>رسیدن به FLOAT ← صفر شدن ساعت</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>۱۲۵</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>وقفهٔ کوتاه</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>شارژ قطع شد ولی کمتر از مهلت وقفه</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>برگشت شارژ ← ادامهٔ شمارش</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>۱۲۶</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>وقفهٔ بلند</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>قطع شارژ بیش از مهلت وقفه</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>صفر شدن ساعت</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>۱۲۶</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>حکم خرابی (قفل)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>رسیدن شمارش به مهلت ۱۲۵</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>فقط تعویض باتری (۳ ثانیه)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>۱۲۵، ۱۲۷، ۱۲۸..۱۳۱</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>قفل + قطع خروجی</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>حکم خرابی و تیک پارامتر ۱۲۷</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>همانند بالا</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>۱۲۷</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F5597"/>
@@ -842,22 +1045,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>تغذیه از باتری</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>حالت اولیهٔ بوت، یا ورودی ضعیف</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>وصل (سطح پایین = روشن)</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
@@ -886,44 +1089,44 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>تغذیه از ورودی</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>ورودی ۵ ثانیه پایدار بالای ۲۲ ولت</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>قطع (سطح بالا = خاموش)</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>بازگشت به باتری</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>ولتاژ ورودی &lt; ۲۱۵۰۰ میلی‌ولت، یا وقفهٔ سخت‌افزاری قطع ورودی</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>وصل</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>آنی (مسیر وقفه)</t>
         </is>
@@ -937,7 +1140,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F5597"/>
@@ -1079,204 +1282,204 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>جدول</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>مرحلهٔ ۰ — بی‌کار</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>چیزی در حال ارسال نیست</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>جدول</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>مرحلهٔ ۱ — BEGIN</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>اعلام تعداد نقاط هر کانال</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>جدول</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>مرحلهٔ ۲ و ۳ — CHUNK</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>نقاط کانال ۱ و کانال ۲ (حداکثر ۲۴ نقطه هر کدام)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>جدول</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>مرحلهٔ ۴ — COMMIT</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>بررسی و نوشتن روی فلش</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>۰ = OK</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>موفق</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>۱ = NO_STAGE</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>کامیت بدون شروع</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>۲ = COUNT</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>تعداد نقاط نامعتبر</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>۳ = MISSING</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>تکه‌ای از نقاط نرسیده است</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>۴ = CHAIN</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>محور زنجیره صعودی نیست</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>۵ = POWER</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>محور توان افت دارد</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>۶ = CRC</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>‏CRC پنل با چیده‌شده نمی‌خواند</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>۷ = FLASH</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>پاک‌کردن یا نوشتن یا بازبینی فلش شکست خورد</t>
         </is>
@@ -1342,162 +1545,162 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>APP_STATE_BOOT</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>حالت اولیه پس از ریست، هنوز تصمیمی گرفته نشده</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>مقدار اولیه در func__Changeover_Init</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>بدون تغییر (محافظ غیرفعال)</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>شارژ تا رسیدن نمونهٔ معتبر شروع نمی‌شود</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>APP_STATE_IDLE</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>مقدار پیش‌فرض متغیر محلی تسک کنترل؛ خروجی ماشین حالت نیست</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>فقط مقداردهی اولیه در task_control.c</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>APP_STATE_INPUT</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>برق ورودی هست و بار از ورودی تغذیه می‌شود</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>نمونه معتبر، بدون خطا، input_present = true</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>غیرفعال (باتری وصل)</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>شارژ مجاز است</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>APP_STATE_BATTERY</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>برق ورودی نیست و بار روی باتری است</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>نمونه معتبر، بدون خطا، input_present = false</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>غیرفعال (باتری وصل)</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>شارژ انجام نمی‌شود (ورودی معتبر نیست)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>APP_STATE_FAULT</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>دست‌کم یک بیت خطا فعال است</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>fault_mask ≠ 0 با نمونهٔ معتبر</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>بدون تغییر (پین دست نمی‌خورد)</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>شارژر به حالت امن می‌رود (SafeIdle)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>APP_STATE_SAFE</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>باتری از خروجی جدا شده است</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>قطع ولتاژ پایین، یا وتوی عدم‌توازن، یا وتوی باتری خراب</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>فعال = باتری قطع</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>شارژر به حالت امن می‌رود</t>
         </is>
@@ -1563,162 +1766,162 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>BOOT</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>INPUT</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>نمونه معتبر و input_present = true</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>اولین نگاشت پس از بوت</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>BOOT</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>BATTERY</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>نمونه معتبر و input_present = false</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>اولین نگاشت پس از بوت</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>همان حالت</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>نمونه NULL یا نامعتبر</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>تصمیمی گرفته نمی‌شود و تایمرها صفر می‌شوند</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>FAULT</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>fault_mask ≠ 0</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>پین محافظ دست نمی‌خورد</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>FAULT</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>INPUT / BATTERY</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>همهٔ بیت‌های خطا پاک شدند</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>نگاشت دوباره از input_present</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>INPUT / BATTERY</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>ولتاژ باتری &lt; ۲۰۸۰۰ میلی‌ولت (قطع بحرانی)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>۳۰۰۰ میلی‌ثانیهٔ پیوسته</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>محافظ فعال می‌شود</t>
         </is>
@@ -1752,81 +1955,81 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>INPUT</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>input_present = true و ولتاژ ≥ ۲۱۲۰۰ میلی‌ولت</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>۳۰۰۰ میلی‌ثانیهٔ پیوسته</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>محافظ غیرفعال و باتری دوباره وصل می‌شود</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>قفل عدم‌توازن + تیک پارامتر ۱۱۷</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>وتوی خروجی سناریوی ۵</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>حکم باتری خراب + تیک پارامتر ۱۲۷</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>وتوی خروجی سناریوی ۶</t>
         </is>
@@ -1913,88 +2116,88 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>CHG_STATE_OFF</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>کانال خاموش و آمادهٔ شروع</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>صفر</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>گذشتن زمان ثبات ۱۵ ثانیه و معتبربودن ورودی ← BULK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>CHG_STATE_BULK</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>جریان ثابت؛ حلقهٔ جریان فرمان می‌دهد</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>از PID، با سقف و حاشیهٔ جریان</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>رسیدن ولتاژ به پنجرهٔ ابزورب ← ABSORB</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>CHG_STATE_ABSORB</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>ولتاژ ثابت؛ حلقهٔ ولتاژ فرمان می‌دهد</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>از PID، زیر سقف ولتاژ</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>افت جریان زیر جریان پایانی، یا سقف زمان ← FLOAT</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>CHG_STATE_FLOAT</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>شارژ تمام شده و کانال پارک است</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>صفر یا نگه‌دارنده</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>افت ولتاژ باتری ← بازگشت به BULK</t>
         </is>
@@ -2067,44 +2270,44 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>CHG_STATE_FINAL_FAULT</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>سه تریپ پیاپی: قفل نهایی کانال</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>صفر و رله باز</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>فقط با ریست برد</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>CHG_STATE_BAT_LOST</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>سیم باتری حین شارژ قطع شده</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>صفر</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>پاک‌شدن بیت خطای قطع باتری ← OFF</t>
         </is>
@@ -2186,66 +2389,66 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>BULK</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>ولتاژ باتری در محدوده به مدت ۱۵ ثانیه و ورودی معتبر</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>شروع نرم از ۱٪ duty</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>BULK</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>ABSORB</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>ولتاژ به پنجرهٔ ابزورب رسید</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>فرمان به حلقهٔ ولتاژ منتقل می‌شود</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>ABSORB</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>FLOAT</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>جریان زیر «جریان پایانی» به مدت پارامتر ۹۶، یا سقف زمان ۹۳</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>اعلام شارژ کامل</t>
         </is>
@@ -2274,22 +2477,22 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>FLOAT</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>BULK</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>افت ولتاژ باتری زیر آستانهٔ شروع دوباره</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>سیکل بعدی شارژ</t>
         </is>
@@ -2340,66 +2543,66 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>JIT_RETRY_WAIT</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>FINAL_FAULT</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>سومین تریپ</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>قفل دائمی کانال + باز شدن رله</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>BAT_LOST</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>ست‌شدن بیت FAULT_CHARGER_BAT_LOST</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>جز FINAL_FAULT که بازنویسی نمی‌شود</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>BAT_LOST</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>پاک‌شدن بیت خطا پس از زمان بازیابی</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>شروع نرم دوباره</t>
         </is>
@@ -2450,22 +2653,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>خروج از مود یا سکوت ۳ ثانیه‌ای لینک</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>duty صفر و بازگشت به خودکار</t>
         </is>
@@ -2486,7 +2689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2531,191 +2734,218 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>۰</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>FAULT_ADC</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>نمونهٔ اندازه‌گیری نامعتبر</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>رسیدن اولین نمونهٔ معتبر (قفل نمی‌شود)</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>سیستم به FAULT و شارژر به حالت امن</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>FAULT_OVERCURRENT_1</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>رزرو — در نسخهٔ فعلی ست نمی‌شود</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>FAULT_OVERCURRENT_2</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>رزرو — در نسخهٔ فعلی ست نمی‌شود</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>۳</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>FAULT_LOW_BATTERY</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>رزرو — از v1.74 تصمیم داخل Changeover است</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>۴</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>FAULT_JITTER_1</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>رزرو — تریپ جیتر در خود شارژر مدیریت می‌شود</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>۵</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>FAULT_JITTER_2</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>رزرو — همانند بالا</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>FAULT_CHARGER_BAT_LOST</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>حالت ۱: نیمِ در حال پمپ بالاتر از آستانهٔ قطع؛ حالت ۲: نیمی زیر ۶ ولت با ورودی سالم — هر دو با دبانس</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>هر دو نیم ≥ ۷ ولت و بدون پمپ، به مدت زمان بازیابی</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>چهرهٔ «قطع باتری» در UI و توقف شارژ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>۷</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>FAULT_CHARGER_TECHNICAL</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>سناریوی ۷: امضای اتصال‌کوتاه (رله باز + PWM واقعی صفر + JIT) یا قطع‌شدن (PWM واقعی &gt;۲۰٪ + جریان صفر)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>فقط reset/power-cycle؛ بیت RAM و latch شارژر با تنظیم پنل پاک نمی‌شود</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>قفل رله/PWM و چهرهٔ سه LED هم‌فاز</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2964,201 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ماشین حالت سناریوی ۷ — خطای فنی طبقهٔ قدرت شارژر</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>حالت</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>شرط ورود</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>خروجی اجباری</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>شرط خروج</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>پارامترهای چهره</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>عادی</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>لچ فنی خاموش و snapshot معتبر</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>رله/PWM طبق کنترل عادی</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>تشخیص یکی از دو امضای فنی</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>اتصال‌کوتاه / سوختن</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>رلهٔ شارژر باز + PWM واقعی = ۰ + JIT ثبت‌شده</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>ست‌کردن FAULT_CHARGER_TECHNICAL؛ هر دو PWM صفر و رله باز</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>فقط reset یا power-cycle</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>۱۳۷..۱۴۲</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>قطع‌شدن / سوختن</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>PWM واقعی &gt;۲۰٪ + جریان شارژ همان کانال = ۰</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>ست‌کردن FAULT_CHARGER_TECHNICAL؛ هر دو PWM صفر و رله باز</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>فقط reset یا power-cycle</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>۱۳۷..۱۴۲</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>قفل فنی</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>FAULT_CHARGER_TECHNICAL یا TechnicalFaultLockout فعال</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>هیچ مسیر عادی، JIT retry، تنظیم پنل یا NVM آن را آزاد نمی‌کند</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>func__Charger_Init پس از reset</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>سه LED هم‌زمان؛ بوق مستقل</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>چهرهٔ UI</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>بیت ۷ در Ui_Tick قبل از OverVoltage بررسی می‌شود</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>هر سه LED از یک phase و duty مشترک؛ بوق q137..q140</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>پاک‌شدن بیت پس از reset</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>q141..q142</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2779,243 +3203,270 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>نمونهٔ نامعتبر</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>snapshot برابر NULL یا valid = false</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>همهٔ چراغ‌ها خاموش</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>۰ (بالاترین)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>خطای فنی برد (سناریو ۷)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>FAULT_CHARGER_TECHNICAL قفل است</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>هر سه LED هم‌زمان با phase مشترک</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>بوق مستقل ۱۳۷..۱۴۰</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>اضافه‌ولتاژ ورودی</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>ولتاژ ورودی بالای آستانهٔ ۷۰ با هیسترزیس ۷۱</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>قرمز چشمک‌زن + سبز روشن</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>بوق دوره‌ای (۴۰..۴۳)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>قطع باتری</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>بیت FAULT_CHARGER_BAT_LOST قفل است</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>چهرهٔ قطع باتری</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>سه بوق کوتاه (۴۷..۴۹)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>۳</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>باتری خراب (سناریو ۶)</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>حکم مهلت شارژ قفل شده</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>قرمز ثابت (پیش‌فرض)</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>بوق هر ۱۰ دقیقه به طول ۱۲۰ms</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>۴</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>عدم‌توازن (سناریو ۵)</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>قفل عدم‌توازن</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>قرمز ثابت</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>بوق کوتاه دوره‌ای (۱۱۵/۱۱۶)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>۵</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>شارژ کامل</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>اعلام اتمام شارژ یا قفل ولتاژی ۱۰۰/۹۵</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>سبز ثابت</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>ورودی سالم بدون شارژ</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>ورودی هست ولی هیچ کانالی پمپ نمی‌کند</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>سبز ثابت</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>۷</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>در حال شارژ</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>ورودی هست و کانالی فعال است</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>سبز ثابت + زرد چشمک‌زن متناسب با درصد</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>۸</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>کار روی باتری (دشارژ)</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>ورودی قطع است</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>سبز چشمک‌زن متناسب با درصد</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>باندهای بوق ۱ تا ۳ و باند بحرانی</t>
         </is>
@@ -3029,7 +3480,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F5597"/>
@@ -3075,44 +3526,44 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>سنجش‌نشده</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>درون مهلت پس از شروع/پایان شارژ، یا نمونهٔ نامعتبر، یا نبود باتری</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>گذشتن مهلت ۱۱۰/۱۱۱</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>۱۱۰، ۱۱۱</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>سالم</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>اختلاف دو نیم زیر حد</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>عبور اختلاف از حد</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>۱۰۸ (استراحت/شارژ)، ۱۰۹ (دشارژ)</t>
         </is>
@@ -3163,253 +3614,68 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>قفل</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>رسیدن شمارش رویدادها به ۱۱۴</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>فقط تعویض باتری (۳ ثانیه بدون باتری)</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>۱۱۴، ۱۱۵، ۱۱۶، ۱۱۷</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>قفل + قطع خروجی</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>قفل و تیک پارامتر ۱۱۷</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>همانند بالا</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>۱۱۷</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>قفل + توقف شارژ</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>گذشتن ۱۱۸ سیکل شارژ پس از قفل</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>همانند بالا</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>۱۱۸</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="002F5597"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ماشین حالت سناریوی ۶ (مهلت شارژ پیوسته)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>حالت</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>شرط ورود</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>شرط خروج</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>پارامترها</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>شمارش متوقف</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>کانال شارژ نمی‌کند</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>شروع BULK یا ABSORB</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>در حال شمارش</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>کانال در BULK یا ABSORB است</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>رسیدن به FLOAT ← صفر شدن ساعت</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>۱۲۵</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>وقفهٔ کوتاه</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>شارژ قطع شد ولی کمتر از مهلت وقفه</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>برگشت شارژ ← ادامهٔ شمارش</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>۱۲۶</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>وقفهٔ بلند</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>قطع شارژ بیش از مهلت وقفه</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>صفر شدن ساعت</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>۱۲۶</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>حکم خرابی (قفل)</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>رسیدن شمارش به مهلت ۱۲۵</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>فقط تعویض باتری (۳ ثانیه)</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>۱۲۵، ۱۲۷، ۱۲۸..۱۳۱</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>قفل + قطع خروجی</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>حکم خرابی و تیک پارامتر ۱۲۷</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>همانند بالا</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>۱۲۷</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align panel validation with firmware and verify optimistic charger preview
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Machine.xlsx
+++ b/Documentation/System_State_Machine.xlsx
@@ -13,11 +13,12 @@
     <sheet name="۳ حالت شارژر" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="۴ گذار شارژر" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="۵ خطاها" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="۶ چهرهٔ UI" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="۷ عدم‌توازن" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="۸ باتری خراب" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="۹ تغذیهٔ MCU" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="۱۰ لینک ESP" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="۵-الف خطای فنی" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="۶ چهرهٔ UI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="۷ عدم‌توازن" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="۸ باتری خراب" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="۹ تغذیهٔ MCU" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="۱۰ لینک ESP" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -76,6 +77,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
@@ -92,11 +98,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -529,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -647,94 +648,106 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>۶ چهرهٔ UI</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>اولویت سناریوها و چهرهٔ چراغ و بوق</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Firmware/Modules/Ui/ui_led.c</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>۵-الف خطای فنی</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>سناریوی ۷: تشخیص سوختن ترانزیستور، قفل RAM و reset</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/Charger/charger.c، Firmware/Modules/Ui/ui_led.c</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>۷ عدم‌توازن</t>
+          <t>۶ چهرهٔ UI</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>حالت‌های سناریوی ۵</t>
+          <t>اولویت سناریوها و چهرهٔ چراغ و بوق</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Firmware/Modules/Imbalance/imbalance.c</t>
+          <t>Firmware/Modules/Ui/ui_led.c</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>۸ باتری خراب</t>
+          <t>۷ عدم‌توازن</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>حالت‌های سناریوی ۶</t>
+          <t>حالت‌های سناریوی ۵</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>charger.c (DeadBatteryTick)</t>
+          <t>Firmware/Modules/Imbalance/imbalance.c</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>۹ تغذیهٔ MCU</t>
+          <t>۸ باتری خراب</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>مسیر تغذیهٔ خود میکرو</t>
+          <t>حالت‌های سناریوی ۶</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Firmware/Modules/McuPowerPath/mcu_power_path.c</t>
+          <t>charger.c (DeadBatteryTick)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>۹ تغذیهٔ MCU</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>مسیر تغذیهٔ خود میکرو</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/McuPowerPath/mcu_power_path.c</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>۱۰ لینک ESP</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>حالت پارسر و مراحل ارسال جدول</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Firmware/Modules/EspLink/esp_link.c، Firmware/Modules/CalLut/cal_lut.c</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr"/>
@@ -742,47 +755,52 @@
       <c r="C14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>نسخهٔ ماژولی</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>همین حالت‌ها، ماژول‌به‌ماژول و کنار برگهٔ اعتبارسنجی همان ماژول: Firmware/Modules/&lt;نام&gt;/&lt;نام&gt;_State_Machine.xlsx — برای کار روی میز تست از این‌ها استفاده کنید، این کتاب نمای سیستمی است</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>tools/make_module_state_machines.py</t>
-        </is>
-      </c>
+      <c r="A15" s="6" t="inlineStr"/>
+      <c r="B15" s="6" t="inlineStr"/>
+      <c r="C15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
+          <t>نسخهٔ ماژولی</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>همین حالت‌ها، ماژول‌به‌ماژول و کنار برگهٔ اعتبارسنجی همان ماژول: Firmware/Modules/&lt;نام&gt;/&lt;نام&gt;_State_Machine.xlsx — برای کار روی میز تست از این‌ها استفاده کنید، این کتاب نمای سیستمی است</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>tools/make_module_state_machines.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
           <t>رنگ‌ها</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>سبز = عادی/سالم · زرد = هشدار یا انتظار · قرمز = خطا یا قفل · نارنجی = در حال کار · خاکستری = بی‌کار · آبی = اطلاعاتی</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>بازتولید</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>python3 tools/make_state_machine_xlsx.py</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>tools/make_state_machine_xlsx.py</t>
         </is>
@@ -797,6 +815,191 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ماشین حالت سناریوی ۶ (مهلت شارژ پیوسته)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>حالت</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>شرط ورود</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>شرط خروج</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>پارامترها</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>شمارش متوقف</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>کانال شارژ نمی‌کند</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>شروع BULK یا ABSORB</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>در حال شمارش</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>کانال در BULK یا ABSORB است</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>رسیدن به FLOAT ← صفر شدن ساعت</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>۱۲۵</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>وقفهٔ کوتاه</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>شارژ قطع شد ولی کمتر از مهلت وقفه</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>برگشت شارژ ← ادامهٔ شمارش</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>۱۲۶</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>وقفهٔ بلند</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>قطع شارژ بیش از مهلت وقفه</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>صفر شدن ساعت</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>۱۲۶</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>حکم خرابی (قفل)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>رسیدن شمارش به مهلت ۱۲۵</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>فقط تعویض باتری (۳ ثانیه)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>۱۲۵، ۱۲۷، ۱۲۸..۱۳۱</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>قفل + قطع خروجی</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>حکم خرابی و تیک پارامتر ۱۲۷</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>همانند بالا</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>۱۲۷</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F5597"/>
@@ -842,22 +1045,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>تغذیه از باتری</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>حالت اولیهٔ بوت، یا ورودی ضعیف</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>وصل (سطح پایین = روشن)</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
@@ -886,44 +1089,44 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>تغذیه از ورودی</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>ورودی ۵ ثانیه پایدار بالای ۲۲ ولت</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>قطع (سطح بالا = خاموش)</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>بازگشت به باتری</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>ولتاژ ورودی &lt; ۲۱۵۰۰ میلی‌ولت، یا وقفهٔ سخت‌افزاری قطع ورودی</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>وصل</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>آنی (مسیر وقفه)</t>
         </is>
@@ -937,7 +1140,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F5597"/>
@@ -1079,204 +1282,204 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>جدول</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>مرحلهٔ ۰ — بی‌کار</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>چیزی در حال ارسال نیست</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>جدول</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>مرحلهٔ ۱ — BEGIN</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>اعلام تعداد نقاط هر کانال</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>جدول</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>مرحلهٔ ۲ و ۳ — CHUNK</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>نقاط کانال ۱ و کانال ۲ (حداکثر ۲۴ نقطه هر کدام)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>جدول</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>مرحلهٔ ۴ — COMMIT</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>بررسی و نوشتن روی فلش</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>۰ = OK</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>موفق</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>۱ = NO_STAGE</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>کامیت بدون شروع</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>۲ = COUNT</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>تعداد نقاط نامعتبر</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>۳ = MISSING</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>تکه‌ای از نقاط نرسیده است</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>۴ = CHAIN</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>محور زنجیره صعودی نیست</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>۵ = POWER</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>محور توان افت دارد</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>۶ = CRC</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>‏CRC پنل با چیده‌شده نمی‌خواند</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>کد وضعیت</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>۷ = FLASH</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>پاک‌کردن یا نوشتن یا بازبینی فلش شکست خورد</t>
         </is>
@@ -1342,162 +1545,162 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>APP_STATE_BOOT</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>حالت اولیه پس از ریست، هنوز تصمیمی گرفته نشده</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>مقدار اولیه در func__Changeover_Init</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>بدون تغییر (محافظ غیرفعال)</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>شارژ تا رسیدن نمونهٔ معتبر شروع نمی‌شود</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>APP_STATE_IDLE</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>مقدار پیش‌فرض متغیر محلی تسک کنترل؛ خروجی ماشین حالت نیست</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>فقط مقداردهی اولیه در task_control.c</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>APP_STATE_INPUT</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>برق ورودی هست و بار از ورودی تغذیه می‌شود</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>نمونه معتبر، بدون خطا، input_present = true</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>غیرفعال (باتری وصل)</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>شارژ مجاز است</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>APP_STATE_BATTERY</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>برق ورودی نیست و بار روی باتری است</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>نمونه معتبر، بدون خطا، input_present = false</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>غیرفعال (باتری وصل)</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>شارژ انجام نمی‌شود (ورودی معتبر نیست)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>APP_STATE_FAULT</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>دست‌کم یک بیت خطا فعال است</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>fault_mask ≠ 0 با نمونهٔ معتبر</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>بدون تغییر (پین دست نمی‌خورد)</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>شارژر به حالت امن می‌رود (SafeIdle)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>APP_STATE_SAFE</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>باتری از خروجی جدا شده است</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>قطع ولتاژ پایین، یا وتوی عدم‌توازن، یا وتوی باتری خراب</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>فعال = باتری قطع</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>شارژر به حالت امن می‌رود</t>
         </is>
@@ -1563,162 +1766,162 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>BOOT</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>INPUT</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>نمونه معتبر و input_present = true</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>اولین نگاشت پس از بوت</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>BOOT</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>BATTERY</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>نمونه معتبر و input_present = false</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>اولین نگاشت پس از بوت</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>همان حالت</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>نمونه NULL یا نامعتبر</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>تصمیمی گرفته نمی‌شود و تایمرها صفر می‌شوند</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>FAULT</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>fault_mask ≠ 0</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>پین محافظ دست نمی‌خورد</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>FAULT</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>INPUT / BATTERY</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>همهٔ بیت‌های خطا پاک شدند</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>نگاشت دوباره از input_present</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>INPUT / BATTERY</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>ولتاژ باتری &lt; ۲۰۸۰۰ میلی‌ولت (قطع بحرانی)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>۳۰۰۰ میلی‌ثانیهٔ پیوسته</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>محافظ فعال می‌شود</t>
         </is>
@@ -1752,81 +1955,81 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>INPUT</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>input_present = true و ولتاژ ≥ ۲۱۲۰۰ میلی‌ولت</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>۳۰۰۰ میلی‌ثانیهٔ پیوسته</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>محافظ غیرفعال و باتری دوباره وصل می‌شود</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>قفل عدم‌توازن + تیک پارامتر ۱۱۷</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>وتوی خروجی سناریوی ۵</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>حکم باتری خراب + تیک پارامتر ۱۲۷</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>وتوی خروجی سناریوی ۶</t>
         </is>
@@ -1913,88 +2116,88 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>CHG_STATE_OFF</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>کانال خاموش و آمادهٔ شروع</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>صفر</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>گذشتن زمان ثبات ۱۵ ثانیه و معتبربودن ورودی ← BULK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>CHG_STATE_BULK</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>جریان ثابت؛ حلقهٔ جریان فرمان می‌دهد</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>از PID، با سقف و حاشیهٔ جریان</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>رسیدن ولتاژ به پنجرهٔ ابزورب ← ABSORB</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>CHG_STATE_ABSORB</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>ولتاژ ثابت؛ حلقهٔ ولتاژ فرمان می‌دهد</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>از PID، زیر سقف ولتاژ</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>افت جریان زیر جریان پایانی، یا سقف زمان ← FLOAT</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>CHG_STATE_FLOAT</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>شارژ تمام شده و کانال پارک است</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>صفر یا نگه‌دارنده</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>افت ولتاژ باتری ← بازگشت به BULK</t>
         </is>
@@ -2067,44 +2270,44 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>CHG_STATE_FINAL_FAULT</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>سه تریپ پیاپی: قفل نهایی کانال</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>صفر و رله باز</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>فقط با ریست برد</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>CHG_STATE_BAT_LOST</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>سیم باتری حین شارژ قطع شده</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>صفر</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>پاک‌شدن بیت خطای قطع باتری ← OFF</t>
         </is>
@@ -2186,66 +2389,66 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>BULK</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>ولتاژ باتری در محدوده به مدت ۱۵ ثانیه و ورودی معتبر</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>شروع نرم از ۱٪ duty</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>BULK</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>ABSORB</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>ولتاژ به پنجرهٔ ابزورب رسید</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>فرمان به حلقهٔ ولتاژ منتقل می‌شود</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>ABSORB</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>FLOAT</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>جریان زیر «جریان پایانی» به مدت پارامتر ۹۶، یا سقف زمان ۹۳</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>اعلام شارژ کامل</t>
         </is>
@@ -2274,22 +2477,22 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>FLOAT</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>BULK</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>افت ولتاژ باتری زیر آستانهٔ شروع دوباره</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>سیکل بعدی شارژ</t>
         </is>
@@ -2340,66 +2543,66 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>JIT_RETRY_WAIT</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>FINAL_FAULT</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>سومین تریپ</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>قفل دائمی کانال + باز شدن رله</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>BAT_LOST</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>ست‌شدن بیت FAULT_CHARGER_BAT_LOST</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>جز FINAL_FAULT که بازنویسی نمی‌شود</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>BAT_LOST</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>پاک‌شدن بیت خطا پس از زمان بازیابی</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>شروع نرم دوباره</t>
         </is>
@@ -2450,22 +2653,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>خروج از مود یا سکوت ۳ ثانیه‌ای لینک</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>duty صفر و بازگشت به خودکار</t>
         </is>
@@ -2486,7 +2689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2531,191 +2734,218 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>۰</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>FAULT_ADC</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>نمونهٔ اندازه‌گیری نامعتبر</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>رسیدن اولین نمونهٔ معتبر (قفل نمی‌شود)</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>سیستم به FAULT و شارژر به حالت امن</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>FAULT_OVERCURRENT_1</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>رزرو — در نسخهٔ فعلی ست نمی‌شود</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>FAULT_OVERCURRENT_2</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>رزرو — در نسخهٔ فعلی ست نمی‌شود</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>۳</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>FAULT_LOW_BATTERY</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>رزرو — از v1.74 تصمیم داخل Changeover است</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>۴</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>FAULT_JITTER_1</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>رزرو — تریپ جیتر در خود شارژر مدیریت می‌شود</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>۵</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>FAULT_JITTER_2</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>رزرو — همانند بالا</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>FAULT_CHARGER_BAT_LOST</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>حالت ۱: نیمِ در حال پمپ بالاتر از آستانهٔ قطع؛ حالت ۲: نیمی زیر ۶ ولت با ورودی سالم — هر دو با دبانس</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>هر دو نیم ≥ ۷ ولت و بدون پمپ، به مدت زمان بازیابی</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>چهرهٔ «قطع باتری» در UI و توقف شارژ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>۷</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>FAULT_CHARGER_TECHNICAL</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>سناریوی ۷: امضای اتصال‌کوتاه (رله باز + PWM واقعی صفر + JIT) یا قطع‌شدن (PWM واقعی &gt;۲۰٪ + جریان صفر)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>فقط reset/power-cycle؛ بیت RAM و latch شارژر با تنظیم پنل پاک نمی‌شود</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>قفل رله/PWM و چهرهٔ سه LED هم‌فاز</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2964,201 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ماشین حالت سناریوی ۷ — خطای فنی طبقهٔ قدرت شارژر</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>حالت</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>شرط ورود</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>خروجی اجباری</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>شرط خروج</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>پارامترهای چهره</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>عادی</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>لچ فنی خاموش و snapshot معتبر</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>رله/PWM طبق کنترل عادی</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>تشخیص یکی از دو امضای فنی</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>اتصال‌کوتاه / سوختن</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>رلهٔ شارژر باز + PWM واقعی = ۰ + JIT ثبت‌شده</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>ست‌کردن FAULT_CHARGER_TECHNICAL؛ هر دو PWM صفر و رله باز</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>فقط reset یا power-cycle</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>۱۳۷..۱۴۲</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>قطع‌شدن / سوختن</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>PWM واقعی &gt;۲۰٪ + جریان شارژ همان کانال = ۰</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>ست‌کردن FAULT_CHARGER_TECHNICAL؛ هر دو PWM صفر و رله باز</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>فقط reset یا power-cycle</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>۱۳۷..۱۴۲</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>قفل فنی</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>FAULT_CHARGER_TECHNICAL یا TechnicalFaultLockout فعال</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>هیچ مسیر عادی، JIT retry، تنظیم پنل یا NVM آن را آزاد نمی‌کند</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>func__Charger_Init پس از reset</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>سه LED هم‌زمان؛ بوق مستقل</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>چهرهٔ UI</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>بیت ۷ در Ui_Tick قبل از OverVoltage بررسی می‌شود</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>هر سه LED از یک phase و duty مشترک؛ بوق q137..q140</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>پاک‌شدن بیت پس از reset</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>q141..q142</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2779,243 +3203,270 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>نمونهٔ نامعتبر</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>snapshot برابر NULL یا valid = false</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>همهٔ چراغ‌ها خاموش</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>۰ (بالاترین)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>خطای فنی برد (سناریو ۷)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>FAULT_CHARGER_TECHNICAL قفل است</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>هر سه LED هم‌زمان با phase مشترک</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>بوق مستقل ۱۳۷..۱۴۰</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>اضافه‌ولتاژ ورودی</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>ولتاژ ورودی بالای آستانهٔ ۷۰ با هیسترزیس ۷۱</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>قرمز چشمک‌زن + سبز روشن</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>بوق دوره‌ای (۴۰..۴۳)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>قطع باتری</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>بیت FAULT_CHARGER_BAT_LOST قفل است</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>چهرهٔ قطع باتری</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>سه بوق کوتاه (۴۷..۴۹)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>۳</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>باتری خراب (سناریو ۶)</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>حکم مهلت شارژ قفل شده</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>قرمز ثابت (پیش‌فرض)</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>بوق هر ۱۰ دقیقه به طول ۱۲۰ms</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>۴</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>عدم‌توازن (سناریو ۵)</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>قفل عدم‌توازن</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>قرمز ثابت</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>بوق کوتاه دوره‌ای (۱۱۵/۱۱۶)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>۵</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>شارژ کامل</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>اعلام اتمام شارژ یا قفل ولتاژی ۱۰۰/۹۵</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>سبز ثابت</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>ورودی سالم بدون شارژ</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>ورودی هست ولی هیچ کانالی پمپ نمی‌کند</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>سبز ثابت</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>۷</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>در حال شارژ</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>ورودی هست و کانالی فعال است</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>سبز ثابت + زرد چشمک‌زن متناسب با درصد</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>۸</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>کار روی باتری (دشارژ)</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>ورودی قطع است</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>سبز چشمک‌زن متناسب با درصد</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>باندهای بوق ۱ تا ۳ و باند بحرانی</t>
         </is>
@@ -3029,7 +3480,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F5597"/>
@@ -3075,44 +3526,44 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>سنجش‌نشده</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>درون مهلت پس از شروع/پایان شارژ، یا نمونهٔ نامعتبر، یا نبود باتری</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>گذشتن مهلت ۱۱۰/۱۱۱</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>۱۱۰، ۱۱۱</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>سالم</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>اختلاف دو نیم زیر حد</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>عبور اختلاف از حد</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>۱۰۸ (استراحت/شارژ)، ۱۰۹ (دشارژ)</t>
         </is>
@@ -3163,253 +3614,68 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>قفل</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>رسیدن شمارش رویدادها به ۱۱۴</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>فقط تعویض باتری (۳ ثانیه بدون باتری)</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>۱۱۴، ۱۱۵، ۱۱۶، ۱۱۷</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>قفل + قطع خروجی</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>قفل و تیک پارامتر ۱۱۷</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>همانند بالا</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>۱۱۷</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>قفل + توقف شارژ</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>گذشتن ۱۱۸ سیکل شارژ پس از قفل</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>همانند بالا</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>۱۱۸</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="002F5597"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ماشین حالت سناریوی ۶ (مهلت شارژ پیوسته)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>حالت</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>شرط ورود</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>شرط خروج</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>پارامترها</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>شمارش متوقف</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>کانال شارژ نمی‌کند</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>شروع BULK یا ABSORB</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>در حال شمارش</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>کانال در BULK یا ABSORB است</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>رسیدن به FLOAT ← صفر شدن ساعت</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>۱۲۵</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>وقفهٔ کوتاه</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>شارژ قطع شد ولی کمتر از مهلت وقفه</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>برگشت شارژ ← ادامهٔ شمارش</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>۱۲۶</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>وقفهٔ بلند</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>قطع شارژ بیش از مهلت وقفه</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>صفر شدن ساعت</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>۱۲۶</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>حکم خرابی (قفل)</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>رسیدن شمارش به مهلت ۱۲۵</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>فقط تعویض باتری (۳ ثانیه)</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>۱۲۵، ۱۲۷، ۱۲۸..۱۳۱</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>قفل + قطع خروجی</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>حکم خرابی و تیک پارامتر ۱۲۷</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>همانند بالا</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>۱۲۷</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs/workbooks review: status-code tables match cal_lut.h (5=DIP, 8=RANGE); validation sheets use counts/BatteryMa; Program_Map regenerated; stale Vin/Vbat ETA comment removed from measurement.h
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Machine.xlsx
+++ b/Documentation/System_State_Machine.xlsx
@@ -1147,7 +1147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1442,12 +1442,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>۵ = POWER</t>
+          <t>۵ = DIP</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>محور توان افت دارد</t>
+          <t>جریان باتری افت دارد</t>
         </is>
       </c>
     </row>
@@ -1482,6 +1482,23 @@
       <c r="C20" s="4" t="inlineStr">
         <is>
           <t>پاک‌کردن یا نوشتن یا بازبینی فلش شکست خورد</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>کد وضعیت</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>۸ = RANGE</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>شمارش بالاتر از ADC ۱۲ بیتی (۴۰۹۵)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(audit): full-program line audit - Vazirmatn everywhere, two latent overflows closed
- All 15 validation/state workbooks: every cell now Vazirmatn
  (29,169 cells; size/bold/colour/underline preserved). The ESP
  panel already served Vazirmatn.
- ui_led.c BatteryRun: green min-off (id 67) and period (id 66) are
  clamped independently, so min-off could exceed the whole period
  and the on-time subtraction underflowed to a ~49-day green phase.
  Clamp off-time to the period first (same pattern as yellow).
- plink_link.h bench statistics: saturate the 60000-frame sum
  instead of wrapping it (a near-ceiling field such as the
  dead-battery elapsed counter could corrupt the average).

Audit covered Firmware (App/Rtos/Bsp/all modules), both ESP
panels' link/http layers line by line; no other defect found.
Both gates green; flash 48,544 B (+8), RAM budget OK.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Machine.xlsx
+++ b/Documentation/System_State_Machine.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,13 @@
     <font>
       <name val="Vazirmatn"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Vazirmatn"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -132,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -164,6 +171,7 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -544,6 +552,8 @@
           <t>ماشین حالت کل برنامه ChangeOver — راهنما و فهرست</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -836,6 +846,9 @@
           <t>ماشین حالت سناریوی ۶ (مهلت شارژ پیوسته)</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1021,6 +1034,9 @@
           <t>مسیر تغذیهٔ خود میکرو (Q1 روی PB5)</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1161,6 +1177,8 @@
           <t>حالت پارسر فریم و مراحل انتقال جدول کالیبراسیون</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1533,6 +1551,10 @@
           <t>حالت‌های اصلی سیستم (app_state_t)</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1754,6 +1776,10 @@
           <t>گذارهای حالت سیستم — شرط و زمان</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -2109,6 +2135,9 @@
           <t>حالت‌های هر کانال شارژ (charger_state_t)</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -2382,6 +2411,9 @@
           <t>گذارهای کانال شارژ</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -2722,6 +2754,10 @@
           <t>بیت‌های خطا (fault_mask_t)</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -2997,6 +3033,10 @@
           <t>ماشین حالت سناریوی ۷ — خطای فنی طبقهٔ قدرت شارژر</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -3191,6 +3231,10 @@
           <t>اولویت سناریوهای چراغ و بوق (func__Ui_Tick)</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -3519,6 +3563,9 @@
           <t>ماشین حالت سناریوی ۵ (عدم‌توازن دو نیمِ باتری)</t>
         </is>
       </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Reconnect output after a qualified battery swap without mains
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Machine.xlsx
+++ b/Documentation/System_State_Machine.xlsx
@@ -1719,7 +1719,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>شارژر به حالت امن می‌رود</t>
+          <t>در صورت حضور ورودی معتبر، شارژ مطابق گیت‌های سناریوی ۵/۶ مجاز است</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1999,29 +1999,29 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>هر حالت</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>قفل عدم‌توازن + تیک پارامتر ۱۱۷</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>آنی</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>وتوی خروجی سناریوی ۵</t>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>BATTERY</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>تعویض باتری تأییدشده (نبود پیوستهٔ باتری) و ولتاژ ≥ ۲۱۲۰۰ میلی‌ولت</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>۳۰۰۰ میلی‌ثانیه نبود + ۳۰۰۰ میلی‌ثانیهٔ پیوسته</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>استثنای ۲۰۲۶-۱۰-۲۳: بدون برق شهر هم وصل می‌شود</t>
         </is>
       </c>
     </row>
@@ -2038,44 +2038,71 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
+          <t>قفل عدم‌توازن + تیک پارامتر ۱۱۷</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>آنی</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>وتوی خروجی سناریوی ۵</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>هر حالت</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
           <t>حکم باتری خراب + تیک پارامتر ۱۲۷</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>وتوی خروجی سناریوی ۶</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>ورودی قطع است</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>ورودی قطع است و باتری هم جدا نشده</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>بدون ورودی، وصل مجدد انجام نمی‌شود (تصمیم تأییدشدهٔ کاربر)</t>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>بدون ورودی و بدون تعویض باتری، وصل مجدد انجام نمی‌شود (تصمیم ۲۰۲۶-۱۰-۰۶)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reconnect a recovered pack without mains after a 10 s healthy hold
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Machine.xlsx
+++ b/Documentation/System_State_Machine.xlsx
@@ -1738,7 +1738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2011,17 +2011,17 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>تعویض باتری تأییدشده (نبود پیوستهٔ باتری) و ولتاژ ≥ ۲۱۲۰۰ میلی‌ولت</t>
+          <t>ولتاژ سالم و پیوسته ≥ ۲۱۲۰۰ میلی‌ولت بدون برق شهر (بازیابی یا تعویض باتری)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>۳۰۰۰ میلی‌ثانیه نبود + ۳۰۰۰ میلی‌ثانیهٔ پیوسته</t>
+          <t>۱۰۰۰۰ میلی‌ثانیهٔ پیوسته + ۳۰۰۰ میلی‌ثانیه</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>استثنای ۲۰۲۶-۱۰-۲۳: بدون برق شهر هم وصل می‌شود</t>
+          <t>استثنای ۲۰۲۶-۱۰-۲۳، با محافظ چرخهٔ ۶۰ ثانیه</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>ورودی قطع است و باتری هم جدا نشده</t>
+          <t>ورودی قطع است و ولتاژ سالم کمتر از ۱۰ ثانیه پیوسته مانده</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -2102,7 +2102,34 @@
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>بدون ورودی و بدون تعویض باتری، وصل مجدد انجام نمی‌شود (تصمیم ۲۰۲۶-۱۰-۰۶)</t>
+          <t>بدون برق شهر و بدون پنجرهٔ سالمِ کامل، وصل انجام نمی‌شود</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>بعد از وصلِ بدون برق شهر، قطع دوباره ظرف ۶۰ ثانیه</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>محافظ چرخه: تا برگشت برق شهر وصل خودکار انجام نمی‌شود</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: bring the manual, both workbooks and the READMEs to the final v1.90 battery-run rules
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Machine.xlsx
+++ b/Documentation/System_State_Machine.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="۱ حالت سیستم" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="۲ گذار سیستم" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="۳ حالت شارژر" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="۴ گذار شارژر" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="۵ خطاها" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="۵-الف خطای فنی" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="۶ چهرهٔ UI" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="۷ عدم‌توازن" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="۸ باتری خراب" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="۸-الف باتری ضعیف" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="۹ تغذیهٔ MCU" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="۱۰ لینک ESP" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۱ حالت سیستم" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۲ گذار سیستم" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۳ حالت شارژر" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۴ گذار شارژر" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۵ خطاها" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۵-الف خطای فنی" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۶ چهرهٔ UI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۷ عدم‌توازن" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۸ باتری خراب" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۸-الف باتری ضعیف" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۹ تغذیهٔ MCU" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="۱۰ لینک ESP" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -724,7 +724,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>سناریوی ۸: حکم، بسته‌ماندن خروجی و پاک‌شدن</t>
+          <t>سناریوی ۸: حکم باتری فرسوده، سقف یک تلاش، آستانهٔ استراحت ۲۵٬۰۰۰ میلی‌ولت و پاک‌شدن</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1024,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1086,147 +1086,255 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>قطعِ داخل پنجرهٔ محافظ بعد از وصلِ بدون برق شهر</t>
+          <t>قطعِ داخل پنجرهٔ محافظ بعد از وصلِ بدون برق شهر یا استراحت زیر آستانه</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>۱۴۹</t>
+          <t>۱۴۹، ۱۶۵</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>حکم قفل شد</t>
+          <t>قطع ولتاژ پایین</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>قطع دوباره داخل ۱۴۹ بعد از وصلِ بدون برق شهر و ۱۴۷ ≠ ۰</t>
+          <t>ولتاژ زیر ۲۱۰۰۰ به‌مدت ۳۰۰۰ میلی‌ثانیه</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>قطع (با ۱۵۷ = ۱) و APP_STATE_SAFE</t>
+          <t>قطع؛ تا برگشت برق ورودی</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>۱۴۷ = ۰ یا استراحت کامل</t>
+          <t>برگشت برق ورودی</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>۱۴۷، ۱۴۹، ۱۵۷</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>استراحت پایین (دشارژ)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>استراحت زیر ۱۶۵ (مثلاً ۲۳٬۰۰۰ میلی‌ولت)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>قطع می‌ماند؛ هیچ تلاشی نمی‌شود</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>رسیدن استراحت به ۱۶۵ یا برگشت برق ورودی</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>۱۶۵</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>استراحت بالا</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>استراحت ≥ ۱۶۵ و ولتاژ سالم پیوسته ≥ ۲۱۲۰۰</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>یک بار بدون برق شهر وصل می‌شود</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>قطع دوباره داخل ۱۴۹</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>۱۶۵، ۱۵۰</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>حکم قفل شد</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>قطع دوباره داخل ۱۴۹ بعد از همان یک وصل و ۱۴۷ ≠ ۰</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>قطع (با ۱۵۷ = ۱) و APP_STATE_SAFE</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>۱۴۷ = ۰ یا استراحت کامل</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>۱۴۷، ۱۴۹، ۱۵۷</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
           <t>چهره در قفل</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>حکم قفل است</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>بی‌ربط به خروجی؛ UI فقط رسم می‌کند</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>پاک‌شدن حکم</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>حکم قفل است و برق ورودی نیست</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>بی‌ربط به خروجی؛ UI فقط بدون برق ورودی رسم می‌کند</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>برگشت برق ورودی (چهره) یا پاک‌شدن حکم</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>۱۵۱..۱۵۶</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>استراحت</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>استراحت سالم</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>حکم قفل و ولتاژ سالم پیوسته ≥ ۲۱۲۰۰ میلی‌ولت</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>قطع می‌ماند</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>پایان ۱۴۸ یا ۱۴۷ = ۰</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>۱۴۸</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>یک تلاش مجدد</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>پایان استراحت</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>پایان استراحت یا دکمهٔ ریست پنل (شناسهٔ ۲۰۴)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>یک بار وصل بدون برق شهر مجاز</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>قطع دوباره ← حکم از نو</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>۱۴۸، ۱۵۰</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>۱۴۸، ۱۵۰، ۲۰۴</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>پاک‌شدن</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>۱۴۷ = ۰ یا پایان استراحت</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>حکم و چهره خاموش</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>قطع دوباره</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>۱۴۷، ۱۴۸</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>قطع سیم بدون برق ورودی</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ولتاژ خوانده‌شده ≈ صفر</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>قطع، همهٔ چراغ‌ها و بوق خاموش، بدون حکم</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>برگشت برق ورودی</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1977,7 +2085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2250,7 +2358,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>ولتاژ سالم و پیوسته ≥ ۲۱۲۰۰ میلی‌ولت بدون برق شهر (بازیابی یا تعویض باتری)</t>
+          <t>استراحت باتری به آستانهٔ پارامتر ۱۶۵ (پیش‌فرض ۲۵٬۰۰۰ میلی‌ولت) رسیده و ولتاژ سالم پیوسته ≥ ۲۱۲۰۰ است، بدون برق شهر</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -2260,7 +2368,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>استثنای ۲۰۲۶-۱۰-۲۳، با محافظ چرخهٔ ۶۰ ثانیه</t>
+          <t>v1.90: زیر آستانهٔ استراحت هیچ وصلِ بدون برق شهری انجام نمی‌شود</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2466,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>بعد از وصلِ بدون برق شهر، قطع دوباره ظرف ۶۰ ثانیه</t>
+          <t>استراحت باتری زیر آستانهٔ ۱۶۵ ماند (مثلاً ۲۳٬۰۰۰ میلی‌ولت)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -2368,59 +2476,113 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>محافظ چرخه: تا برگشت برق شهر وصل خودکار انجام نمی‌شود</t>
+          <t>v1.90: باتری دشارژ است؛ وصل نمی‌شود و حکمی هم زده نمی‌شود</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>بعد از همان یک وصلِ بدون برق شهر، قطع دوباره ظرف ۶۰ ثانیه</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>مسیر تا برگشت برق شهر بسته می‌ماند (سقف تلاش = ۱)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>قطع سیم باتری و برق شهر هم نیست</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>۳۰۰۰ میلی‌ثانیهٔ پیوسته</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>v1.90: سکوت کامل — قطع، همهٔ چراغ‌ها و بوق خاموش، بدون حکم</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>هر حالت</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>حکم باتری ضعیف + تیک پارامتر ۱۵۷ (برق شهر قطع)</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>آنی</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>وتوی خروجی سناریوی ۸: بار روی باتری ضعیف نمی‌رود</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>SAFE (حکم)</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>BATTERY</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>ولتاژ سالم پیوسته ≥ ۲۱۲۰۰ میلی‌ولت به مدت پارامتر ۱۴۸</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>۱۴۸ (پیش‌فرض ۶۰۰۰۰۰) + ۳۰۰۰</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>حکم پاک و فقط یک تلاش مجدد بدون برق شهر</t>
         </is>
@@ -3544,7 +3706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3758,12 +3920,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>باتری ضعیف (سناریو ۸)</t>
+          <t>باتری فرسوده (سناریو ۸)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>حکم باتری ضعیف قفل است</t>
+          <t>حکم قفل است و برق ورودی نیست</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -3778,135 +3940,162 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>۵ب</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>مسیر باتری بسته + بدون برق ورودی</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>ولتاژ پایین قطع کرده یا سقف تلاش تمام شده (پس از سناریو ۸)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>هر سه چراغ خاموش</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>بی‌صدا</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>شارژ کامل</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>اعلام اتمام شارژ یا قفل ولتاژی ۱۰۰/۹۵</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>سبز ثابت</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>۷</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>استراحت حرارتی</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>کانالی یک ساعت نزدیک سقف جریان بوده و ۱۰ دقیقه استراحت می‌کند</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>سبز ثابت + زرد چشمک‌زن ۱ ثانیه‌ای ۵۰٪</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>۸</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>ورودی سالم بدون شارژ</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>ورودی هست ولی هیچ کانالی در حال شارژ نیست</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>سبز ثابت</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>۹</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>در حال شارژ</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>ورودی هست و کانالی فعال است</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>سبز ثابت + زرد چشمک‌زن متناسب با درصد</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>بی‌صدا</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>۱۰</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>کار روی باتری (دشارژ)</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>ورودی قطع است</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>سبز چشمک‌زن متناسب با درصد</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>باندهای بوق ۱ تا ۳ و باند بحرانی</t>
         </is>

</xml_diff>